<commit_message>
feat: initialize frontend with React and Vite
- Added package.json for frontend with dependencies and scripts for development, build, and preview.
- Created App component to display API health status.
- Implemented API client for health check requests.
- Set up main entry point for React application.
- Added basic styles for the application layout.
- Configured Vite for development server.
- Created workspace package.json for managing frontend and backend development scripts.
</commit_message>
<xml_diff>
--- a/imagenes/matricestablas/Tabladecolores.xlsx
+++ b/imagenes/matricestablas/Tabladecolores.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,16 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Número</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Color (RGB)</t>
         </is>
@@ -446,7 +434,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(64, 64, 64, 192)</t>
+          <t>(64, 128, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -456,7 +444,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(128, 64, 64, 192)</t>
+          <t>(128, 128, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -466,7 +454,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>(128, 128, 64, 192)</t>
+          <t>(128, 192, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -476,7 +464,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(128, 128, 128, 192)</t>
+          <t>(192, 192, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -486,7 +474,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>(64, 64, 128, 192)</t>
+          <t>(64, 64, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -496,7 +484,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>(192, 64, 64, 192)</t>
+          <t>(0, 64, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -506,7 +494,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>(64, 128, 128, 192)</t>
+          <t>(64, 64, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -516,7 +504,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>(192, 128, 128, 192)</t>
+          <t>(64, 128, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -526,7 +514,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(192, 192, 192, 192)</t>
+          <t>(128, 128, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -536,7 +524,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>(192, 192, 128, 192)</t>
+          <t>(64, 64, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -546,7 +534,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>(192, 192, 0, 192)</t>
+          <t>(128, 64, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -556,7 +544,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>(64, 128, 64, 192)</t>
+          <t>(192, 128, 192, 192)</t>
         </is>
       </c>
     </row>
@@ -566,7 +554,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(0, 0, 64, 192)</t>
+          <t>(64, 0, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -576,7 +564,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>(0, 0, 0, 192)</t>
+          <t>(0, 0, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -586,7 +574,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>(64, 64, 0, 192)</t>
+          <t>(128, 128, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -596,7 +584,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>(192, 128, 0, 192)</t>
+          <t>(192, 128, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -606,7 +594,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>(0, 64, 64, 192)</t>
+          <t>(192, 64, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -616,7 +604,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>(128, 64, 128, 192)</t>
+          <t>(192, 64, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -626,7 +614,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>(0, 128, 0, 192)</t>
+          <t>(0, 64, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -636,7 +624,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(0, 64, 0, 192)</t>
+          <t>(64, 0, 0, 192)</t>
         </is>
       </c>
     </row>
@@ -646,7 +634,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>(64, 0, 0, 192)</t>
+          <t>(64, 64, 0, 192)</t>
         </is>
       </c>
     </row>
@@ -656,7 +644,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>(128, 128, 0, 192)</t>
+          <t>(128, 64, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -666,7 +654,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>(64, 0, 64, 192)</t>
+          <t>(192, 192, 128, 192)</t>
         </is>
       </c>
     </row>
@@ -676,7 +664,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>(128, 0, 0, 192)</t>
+          <t>(64, 128, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -686,7 +674,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>(128, 128, 192, 192)</t>
+          <t>(128, 128, 0, 192)</t>
         </is>
       </c>
     </row>
@@ -696,7 +684,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>(64, 128, 192, 192)</t>
+          <t>(192, 128, 64, 192)</t>
         </is>
       </c>
     </row>
@@ -706,7 +694,177 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>(128, 192, 192, 192)</t>
+          <t>(128, 64, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>(0, 0, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>(192, 192, 64, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>(192, 0, 64, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>(128, 0, 64, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>(192, 64, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>(128, 0, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>(192, 0, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>(192, 128, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>(192, 192, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>(192, 0, 128, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>(192, 64, 192, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>(0, 64, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>(64, 128, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>(128, 192, 64, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>(128, 192, 0, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>(128, 192, 128, 192)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>(128, 0, 128, 192)</t>
         </is>
       </c>
     </row>

</xml_diff>